<commit_message>
Add double-booking check tests (TC-017, TC-018) — 18/18 PASS
TC-017: POST same room/dates twice via API → verify HTTP 409 and
        "指定の日程はすでに予約済みです" error; UI search confirms
        the booked room is excluded from availability results.

TC-018: Pre-book 雪の間 (room_id=6) via API for 2026-08-22~23,
        then search same dates in UI → verify 雪の間 absent from
        availability list while other rooms remain visible.

Also updates session-test.md with the new test case specs and
second-run results (18 cases, all PASS, ~50s).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test-results.xlsx
+++ b/tests/test-results.xlsx
@@ -21,13 +21,15 @@
     <sheet sheetId="15" name="TC-014" state="visible" r:id="rId18"/>
     <sheet sheetId="16" name="TC-015" state="visible" r:id="rId19"/>
     <sheet sheetId="17" name="TC-016" state="visible" r:id="rId20"/>
+    <sheet sheetId="18" name="TC-017" state="visible" r:id="rId21"/>
+    <sheet sheetId="19" name="TC-018" state="visible" r:id="rId22"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="154">
   <si>
     <t>No.</t>
   </si>
@@ -68,10 +70,10 @@
     <t/>
   </si>
   <si>
-    <t>実施件数: 16件</t>
-  </si>
-  <si>
-    <t>PASS: 16</t>
+    <t>実施件数: 18件</t>
+  </si>
+  <si>
+    <t>PASS: 18</t>
   </si>
   <si>
     <t>FAIL: 0</t>
@@ -80,7 +82,7 @@
     <t>ERROR: 0</t>
   </si>
   <si>
-    <t>実施日: 2026/4/5</t>
+    <t>実施日: 2026/4/6</t>
   </si>
   <si>
     <t>TC-001</t>
@@ -105,7 +107,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:27</t>
+    <t>2026/4/6 16:50:58</t>
   </si>
   <si>
     <t>TC-002</t>
@@ -121,7 +123,7 @@
     <t>"客室一覧" のタイトルと複数の客室カードが表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:28</t>
+    <t>2026/4/6 16:51:00</t>
   </si>
   <si>
     <t>TC-003</t>
@@ -137,7 +139,7 @@
     <t>客室名（松の間）、料金、設備情報が表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:31</t>
+    <t>2026/4/6 16:51:04</t>
   </si>
   <si>
     <t>TC-004</t>
@@ -153,7 +155,7 @@
     <t>"宿泊プラン" のタイトルと複数のプランが表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:34</t>
+    <t>2026/4/6 16:51:07</t>
   </si>
   <si>
     <t>TC-005</t>
@@ -172,7 +174,7 @@
     <t>温泉・施設案内のタイトルとコンテンツが表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:35</t>
+    <t>2026/4/6 16:51:08</t>
   </si>
   <si>
     <t>TC-006</t>
@@ -188,6 +190,9 @@
     <t>"アクセス" タイトルと地図 iframe が表示される</t>
   </si>
   <si>
+    <t>2026/4/6 16:51:09</t>
+  </si>
+  <si>
     <t>TC-007</t>
   </si>
   <si>
@@ -201,7 +206,7 @@
     <t>"お知らせ" タイトルとお知らせ記事が表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:41</t>
+    <t>2026/4/6 16:51:16</t>
   </si>
   <si>
     <t>TC-008</t>
@@ -217,7 +222,7 @@
     <t>"お問い合わせ" タイトルと入力フォームが表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:42</t>
+    <t>2026/4/6 16:51:17</t>
   </si>
   <si>
     <t>TC-009</t>
@@ -234,6 +239,9 @@
   </si>
   <si>
     <t>ステップインジケーター・チェックイン日・チェックアウト日・人数・検索ボタンが表示される</t>
+  </si>
+  <si>
+    <t>2026/4/6 16:51:18</t>
   </si>
   <si>
     <t>TC-010</t>
@@ -250,7 +258,7 @@
     <t>チェックイン日・チェックアウト日のエラーメッセージ「入力してください」が表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:43</t>
+    <t>2026/4/6 16:51:19</t>
   </si>
   <si>
     <t>TC-011</t>
@@ -268,7 +276,7 @@
     <t>空室状況セクションが表示され、利用可能な客室が一覧表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:47</t>
+    <t>2026/4/6 16:51:23</t>
   </si>
   <si>
     <t>TC-012</t>
@@ -285,7 +293,7 @@
     <t>「客室・プランを選択してください」が表示され、プラン選択ボタンが並ぶ</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:52</t>
+    <t>2026/4/6 16:51:28</t>
   </si>
   <si>
     <t>TC-013</t>
@@ -302,7 +310,7 @@
     <t>氏名・メール・電話番号・特別リクエスト欄が表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:50:56</t>
+    <t>2026/4/6 16:51:33</t>
   </si>
   <si>
     <t>TC-014</t>
@@ -319,7 +327,7 @@
     <t>「予約内容をご確認ください」と宿泊情報・お客様情報が表示され、「予約を確定する」ボタンが表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:51:02</t>
+    <t>2026/4/6 16:51:38</t>
   </si>
   <si>
     <t>TC-015</t>
@@ -339,7 +347,7 @@
     <t>「お名前」「メールアドレス」「お問い合わせ内容」のエラーメッセージが表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:51:03</t>
+    <t>2026/4/6 16:51:40</t>
   </si>
   <si>
     <t>TC-016</t>
@@ -357,13 +365,55 @@
     <t>「有効な電話番号を入力してください」のエラーメッセージが表示される</t>
   </si>
   <si>
-    <t>2026/4/5 16:51:09</t>
+    <t>2026/4/6 16:51:46</t>
+  </si>
+  <si>
+    <t>TC-017</t>
+  </si>
+  <si>
+    <t>二重予約チェック</t>
+  </si>
+  <si>
+    <t>二重予約チェック — API 409エラー確認</t>
+  </si>
+  <si>
+    <t>バックエンドサーバー起動済み（localhost:3001）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">① POST /api/reservations で 雪の間(room_id=6) / 2026-08-20〜21 / 1名 の予約を作成
+② 同一の客室・日程で再度 POST
+③ 2回目のレスポンスが HTTP 409 かつ "指定の日程はすでに予約済みです" を返すことを確認
+④ /reserve 画面で同日程を検索し、雪の間が除外されていることをスクリーンショットで記録</t>
+  </si>
+  <si>
+    <t>1回目: HTTP 201 Created / 2回目: HTTP 409 Conflict、error:"指定の日程はすでに予約済みです"</t>
+  </si>
+  <si>
+    <t>2026/4/6 16:51:50</t>
+  </si>
+  <si>
+    <t>TC-018</t>
+  </si>
+  <si>
+    <t>二重予約チェック — 予約済み客室が空室検索から除外される確認</t>
+  </si>
+  <si>
+    <t xml:space="preserve">① API で 雪の間(room_id=6) / 2026-08-22〜23 / 1名 の予約を事前登録
+② /reserve へアクセスし、同じ日程（2026-08-22〜23）・1名で空室検索を実行
+③ 検索結果に「雪の間」が表示されないことを確認
+④ 他の空室客室は引き続き表示されることを確認</t>
+  </si>
+  <si>
+    <t>空室リストに「雪の間」が含まれない。他の未予約客室は正常に表示される</t>
+  </si>
+  <si>
+    <t>2026/4/6 16:51:54</t>
   </si>
   <si>
     <t>TC-001  トップページ表示確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:27  ／  実施時間: 925ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:50:58  ／  実施時間: 2257ms</t>
   </si>
   <si>
     <t>—</t>
@@ -375,91 +425,103 @@
     <t>TC-002  客室一覧ページ表示確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:28  ／  実施時間: 965ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:00  ／  実施時間: 1779ms</t>
   </si>
   <si>
     <t>TC-003  客室詳細ページ表示確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:31  ／  実施時間: 2857ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:04  ／  実施時間: 3427ms</t>
   </si>
   <si>
     <t>TC-004  プラン一覧ページ表示確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:34  ／  実施時間: 2856ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:07  ／  実施時間: 3283ms</t>
   </si>
   <si>
     <t>TC-005  温泉・施設案内ページ表示確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:35  ／  実施時間: 663ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:08  ／  実施時間: 1272ms</t>
   </si>
   <si>
     <t>TC-006  アクセスページ表示確認（地図埋め込み）</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:35  ／  実施時間: 224ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:09  ／  実施時間: 451ms</t>
   </si>
   <si>
     <t>TC-007  お知らせページ表示確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:41  ／  実施時間: 5624ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:16  ／  実施時間: 6514ms</t>
   </si>
   <si>
     <t>TC-008  お問い合わせページ表示確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:42  ／  実施時間: 618ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:17  ／  実施時間: 980ms</t>
   </si>
   <si>
     <t>TC-009  予約フォーム Step1 表示確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:42  ／  実施時間: 644ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:18  ／  実施時間: 829ms</t>
   </si>
   <si>
     <t>TC-010  予約 Step1 バリデーション確認（未入力送信）</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:43  ／  実施時間: 1184ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:19  ／  実施時間: 1523ms</t>
   </si>
   <si>
     <t>TC-011  予約 Step1 空室検索実行確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:47  ／  実施時間: 3688ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:23  ／  実施時間: 3926ms</t>
   </si>
   <si>
     <t>TC-012  予約 Step2 客室・プラン選択確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:52  ／  実施時間: 4262ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:28  ／  実施時間: 4273ms</t>
   </si>
   <si>
     <t>TC-013  予約 Step3 お客様情報入力フォーム確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:50:56  ／  実施時間: 4816ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:33  ／  実施時間: 4847ms</t>
   </si>
   <si>
     <t>TC-014  予約 Step4 確認画面表示確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:51:02  ／  実施時間: 5449ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:38  ／  実施時間: 5621ms</t>
   </si>
   <si>
     <t>TC-015  お問い合わせフォーム バリデーション確認</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:51:03  ／  実施時間: 1195ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:40  ／  実施時間: 1367ms</t>
   </si>
   <si>
     <t>TC-016  電話番号バリデーション確認（不正形式）</t>
   </si>
   <si>
-    <t>テスト結果: PASS  ／  実施日時: 2026/4/5 16:51:09  ／  実施時間: 5399ms</t>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:46  ／  実施時間: 5802ms</t>
+  </si>
+  <si>
+    <t>TC-017  二重予約チェック — API 409エラー確認</t>
+  </si>
+  <si>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:50  ／  実施時間: 4484ms</t>
+  </si>
+  <si>
+    <t>TC-018  二重予約チェック — 予約済み客室が空室検索から除外される確認</t>
+  </si>
+  <si>
+    <t>テスト結果: PASS  ／  実施日時: 2026/4/6 16:51:54  ／  実施時間: 3971ms</t>
   </si>
 </sst>
 </file>
@@ -939,6 +1001,94 @@
 </file>
 
 <file path=xl/drawings/drawing16.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12192000" cy="7715250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing17.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12192000" cy="7715250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing18.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1656,7 +1806,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1781,7 +1931,7 @@
         <v>25</v>
       </c>
       <c r="L5" s="6">
-        <v>925</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="6" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1819,7 +1969,7 @@
         <v>30</v>
       </c>
       <c r="L6" s="6">
-        <v>965</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="7" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1857,7 +2007,7 @@
         <v>35</v>
       </c>
       <c r="L7" s="6">
-        <v>2857</v>
+        <v>3427</v>
       </c>
     </row>
     <row r="8" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1895,7 +2045,7 @@
         <v>40</v>
       </c>
       <c r="L8" s="6">
-        <v>2856</v>
+        <v>3283</v>
       </c>
     </row>
     <row r="9" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1933,7 +2083,7 @@
         <v>46</v>
       </c>
       <c r="L9" s="6">
-        <v>663</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="10" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1968,10 +2118,10 @@
         <v>47</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="L10" s="6">
-        <v>224</v>
+        <v>451</v>
       </c>
     </row>
     <row r="11" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1979,22 +2129,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>24</v>
@@ -2003,13 +2153,13 @@
         <v>12</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L11" s="6">
-        <v>5624</v>
+        <v>6514</v>
       </c>
     </row>
     <row r="12" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2017,22 +2167,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>19</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>43</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>24</v>
@@ -2041,13 +2191,13 @@
         <v>12</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L12" s="6">
-        <v>618</v>
+        <v>980</v>
       </c>
     </row>
     <row r="13" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2055,22 +2205,22 @@
         <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>43</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>24</v>
@@ -2079,13 +2229,13 @@
         <v>12</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="L13" s="6">
-        <v>644</v>
+        <v>829</v>
       </c>
     </row>
     <row r="14" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2093,22 +2243,22 @@
         <v>10</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>43</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>24</v>
@@ -2117,13 +2267,13 @@
         <v>12</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L14" s="6">
-        <v>1184</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="15" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2131,22 +2281,22 @@
         <v>11</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>21</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>24</v>
@@ -2155,13 +2305,13 @@
         <v>12</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L15" s="6">
-        <v>3688</v>
+        <v>3926</v>
       </c>
     </row>
     <row r="16" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2169,22 +2319,22 @@
         <v>12</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>21</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H16" s="8" t="s">
         <v>24</v>
@@ -2193,13 +2343,13 @@
         <v>12</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L16" s="6">
-        <v>4262</v>
+        <v>4273</v>
       </c>
     </row>
     <row r="17" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2207,22 +2357,22 @@
         <v>13</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>21</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H17" s="8" t="s">
         <v>24</v>
@@ -2231,13 +2381,13 @@
         <v>12</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="L17" s="6">
-        <v>4816</v>
+        <v>4847</v>
       </c>
     </row>
     <row r="18" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2245,22 +2395,22 @@
         <v>14</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>21</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>24</v>
@@ -2269,13 +2419,13 @@
         <v>12</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L18" s="6">
-        <v>5449</v>
+        <v>5621</v>
       </c>
     </row>
     <row r="19" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2283,22 +2433,22 @@
         <v>15</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>43</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H19" s="8" t="s">
         <v>24</v>
@@ -2307,13 +2457,13 @@
         <v>12</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="L19" s="6">
-        <v>1195</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="20" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2321,22 +2471,22 @@
         <v>16</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>21</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H20" s="8" t="s">
         <v>24</v>
@@ -2345,13 +2495,89 @@
         <v>12</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L20" s="6">
-        <v>5399</v>
+        <v>5802</v>
+      </c>
+    </row>
+    <row r="21" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" s="6">
+        <v>17</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="L21" s="6">
+        <v>4484</v>
+      </c>
+    </row>
+    <row r="22" ht="55" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="6">
+        <v>18</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="L22" s="6">
+        <v>3971</v>
       </c>
     </row>
   </sheetData>
@@ -2374,7 +2600,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -2386,7 +2612,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -2401,7 +2627,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -2429,7 +2655,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -2443,7 +2669,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -2457,7 +2683,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -2468,7 +2694,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -2565,7 +2791,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -2577,7 +2803,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -2592,7 +2818,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -2620,7 +2846,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -2634,7 +2860,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -2648,7 +2874,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -2659,7 +2885,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -2756,7 +2982,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -2768,7 +2994,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -2783,7 +3009,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -2811,7 +3037,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -2825,7 +3051,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -2839,7 +3065,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -2850,7 +3076,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -2947,7 +3173,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -2959,7 +3185,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -2974,7 +3200,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3002,7 +3228,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -3016,7 +3242,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -3030,7 +3256,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -3041,7 +3267,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -3138,7 +3364,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -3150,7 +3376,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -3165,7 +3391,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3193,7 +3419,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -3207,7 +3433,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -3221,7 +3447,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -3232,7 +3458,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -3329,7 +3555,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -3341,7 +3567,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -3356,7 +3582,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3384,7 +3610,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -3398,7 +3624,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -3412,7 +3638,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -3423,7 +3649,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -3520,7 +3746,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -3532,7 +3758,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -3547,7 +3773,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3575,7 +3801,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -3589,7 +3815,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -3603,7 +3829,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -3614,7 +3840,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -3711,7 +3937,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -3723,7 +3949,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -3738,7 +3964,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3766,7 +3992,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -3780,7 +4006,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -3794,7 +4020,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -3805,7 +4031,389 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="A8:H8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H64"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="8" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>105</v>
+      </c>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+    </row>
+    <row r="5" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="A8:H8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H64"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="8" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+    </row>
+    <row r="5" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -3902,7 +4510,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -3914,7 +4522,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -3985,7 +4593,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -3996,7 +4604,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -4093,7 +4701,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4105,7 +4713,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -4176,7 +4784,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -4187,7 +4795,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -4284,7 +4892,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4296,7 +4904,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -4367,7 +4975,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -4378,7 +4986,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -4475,7 +5083,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4487,7 +5095,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -4558,7 +5166,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -4569,7 +5177,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -4666,7 +5274,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4678,7 +5286,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -4749,7 +5357,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -4760,7 +5368,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -4857,7 +5465,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -4869,7 +5477,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -4940,7 +5548,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -4951,7 +5559,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -5048,7 +5656,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -5060,7 +5668,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -5103,7 +5711,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -5117,7 +5725,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -5131,7 +5739,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -5142,7 +5750,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -5239,7 +5847,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -5251,7 +5859,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -5294,7 +5902,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -5308,7 +5916,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -5322,7 +5930,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -5333,7 +5941,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>

</xml_diff>